<commit_message>
Maßstab auch erkennen, wenn Google Sheets 1:24 als Uhrzeit speichert
- parseScale versteht 1:24, 01:24:00, 1/24 und 24 (ebenso 1:32)
- Vorlage: Maßstab-Spalte als Text formatiert

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4m14j9yimsYZgVXMyWVGU
</commit_message>
<xml_diff>
--- a/docs/GR-Legends-Einstellungen.xlsx
+++ b/docs/GR-Legends-Einstellungen.xlsx
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +99,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1057,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1100,7 +1104,7 @@
           <t>Porsche 911 GT3 Beispiel</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>1:24</t>
         </is>
@@ -1115,257 +1119,1577 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="n"/>
-      <c r="B3" s="7" t="n"/>
+      <c r="B3" s="11" t="n"/>
       <c r="C3" s="7" t="n"/>
       <c r="D3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
-      <c r="B4" s="7" t="n"/>
+      <c r="B4" s="11" t="n"/>
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
-      <c r="B5" s="7" t="n"/>
+      <c r="B5" s="11" t="n"/>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="11" t="n"/>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
-      <c r="B7" s="7" t="n"/>
+      <c r="B7" s="11" t="n"/>
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
-      <c r="B8" s="7" t="n"/>
+      <c r="B8" s="11" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="11" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
-      <c r="B10" s="7" t="n"/>
+      <c r="B10" s="11" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="11" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
-      <c r="B12" s="7" t="n"/>
+      <c r="B12" s="11" t="n"/>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="11" t="n"/>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="8" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="n"/>
+      <c r="B15" s="12" t="n"/>
       <c r="C15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="8" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="n"/>
+      <c r="B17" s="12" t="n"/>
       <c r="C17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="8" t="n"/>
+      <c r="B18" s="12" t="n"/>
       <c r="C18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="n"/>
+      <c r="B19" s="12" t="n"/>
       <c r="C19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="8" t="n"/>
+      <c r="B20" s="12" t="n"/>
       <c r="C20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="8" t="n"/>
+      <c r="B21" s="12" t="n"/>
       <c r="C21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="8" t="n"/>
+      <c r="B22" s="12" t="n"/>
       <c r="C22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="8" t="n"/>
+      <c r="B23" s="12" t="n"/>
       <c r="C23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="8" t="n"/>
+      <c r="B24" s="12" t="n"/>
       <c r="C24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="8" t="n"/>
+      <c r="B25" s="12" t="n"/>
       <c r="C25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="8" t="n"/>
+      <c r="B26" s="12" t="n"/>
       <c r="C26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="8" t="n"/>
+      <c r="B27" s="12" t="n"/>
       <c r="C27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="8" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="8" t="n"/>
+      <c r="B29" s="12" t="n"/>
       <c r="C29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="8" t="n"/>
+      <c r="B30" s="12" t="n"/>
       <c r="C30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="8" t="n"/>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="8" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="8" t="n"/>
+      <c r="B33" s="12" t="n"/>
       <c r="C33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="8" t="n"/>
+      <c r="B34" s="12" t="n"/>
       <c r="C34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="8" t="n"/>
+      <c r="B35" s="12" t="n"/>
       <c r="C35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="8" t="n"/>
+      <c r="B36" s="12" t="n"/>
       <c r="C36" s="8" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="8" t="n"/>
+      <c r="B37" s="12" t="n"/>
       <c r="C37" s="8" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="8" t="n"/>
+      <c r="B38" s="12" t="n"/>
       <c r="C38" s="8" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="8" t="n"/>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="8" t="n"/>
+      <c r="B40" s="12" t="n"/>
       <c r="C40" s="8" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="8" t="n"/>
+      <c r="B41" s="12" t="n"/>
       <c r="C41" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="8" t="n"/>
+      <c r="B42" s="12" t="n"/>
       <c r="C42" s="8" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="8" t="n"/>
+      <c r="B43" s="12" t="n"/>
       <c r="C43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="8" t="n"/>
+      <c r="B44" s="12" t="n"/>
       <c r="C44" s="8" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="8" t="n"/>
+      <c r="B45" s="12" t="n"/>
       <c r="C45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="8" t="n"/>
+      <c r="B46" s="12" t="n"/>
       <c r="C46" s="8" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="8" t="n"/>
+      <c r="B47" s="12" t="n"/>
       <c r="C47" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="8" t="n"/>
+      <c r="B48" s="12" t="n"/>
       <c r="C48" s="8" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="8" t="n"/>
+      <c r="B49" s="12" t="n"/>
       <c r="C49" s="8" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="8" t="n"/>
+      <c r="B50" s="12" t="n"/>
       <c r="C50" s="8" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="8" t="n"/>
+      <c r="B51" s="12" t="n"/>
       <c r="C51" s="8" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="8" t="n"/>
+      <c r="B52" s="12" t="n"/>
       <c r="C52" s="8" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="8" t="n"/>
+      <c r="B53" s="12" t="n"/>
       <c r="C53" s="8" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="8" t="n"/>
+      <c r="B54" s="12" t="n"/>
       <c r="C54" s="8" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="8" t="n"/>
+      <c r="B55" s="12" t="n"/>
       <c r="C55" s="8" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="8" t="n"/>
+      <c r="B56" s="12" t="n"/>
       <c r="C56" s="8" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="8" t="n"/>
+      <c r="B57" s="12" t="n"/>
       <c r="C57" s="8" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="8" t="n"/>
+      <c r="B58" s="12" t="n"/>
       <c r="C58" s="8" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="8" t="n"/>
+      <c r="B59" s="12" t="n"/>
       <c r="C59" s="8" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="8" t="n"/>
+      <c r="B60" s="12" t="n"/>
       <c r="C60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="13" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="13" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="13" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="13" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="13" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="13" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="13" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="13" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="13" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="13" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="13" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="13" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="13" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="13" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="13" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="13" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="13" t="n"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="13" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="13" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="13" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="13" t="n"/>
+    </row>
+    <row r="82">
+      <c r="B82" s="13" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="13" t="n"/>
+    </row>
+    <row r="84">
+      <c r="B84" s="13" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="13" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="13" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="13" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="13" t="n"/>
+    </row>
+    <row r="89">
+      <c r="B89" s="13" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="13" t="n"/>
+    </row>
+    <row r="91">
+      <c r="B91" s="13" t="n"/>
+    </row>
+    <row r="92">
+      <c r="B92" s="13" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="13" t="n"/>
+    </row>
+    <row r="94">
+      <c r="B94" s="13" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="13" t="n"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="13" t="n"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="13" t="n"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="13" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="13" t="n"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="13" t="n"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="13" t="n"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="13" t="n"/>
+    </row>
+    <row r="103">
+      <c r="B103" s="13" t="n"/>
+    </row>
+    <row r="104">
+      <c r="B104" s="13" t="n"/>
+    </row>
+    <row r="105">
+      <c r="B105" s="13" t="n"/>
+    </row>
+    <row r="106">
+      <c r="B106" s="13" t="n"/>
+    </row>
+    <row r="107">
+      <c r="B107" s="13" t="n"/>
+    </row>
+    <row r="108">
+      <c r="B108" s="13" t="n"/>
+    </row>
+    <row r="109">
+      <c r="B109" s="13" t="n"/>
+    </row>
+    <row r="110">
+      <c r="B110" s="13" t="n"/>
+    </row>
+    <row r="111">
+      <c r="B111" s="13" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="13" t="n"/>
+    </row>
+    <row r="113">
+      <c r="B113" s="13" t="n"/>
+    </row>
+    <row r="114">
+      <c r="B114" s="13" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="13" t="n"/>
+    </row>
+    <row r="116">
+      <c r="B116" s="13" t="n"/>
+    </row>
+    <row r="117">
+      <c r="B117" s="13" t="n"/>
+    </row>
+    <row r="118">
+      <c r="B118" s="13" t="n"/>
+    </row>
+    <row r="119">
+      <c r="B119" s="13" t="n"/>
+    </row>
+    <row r="120">
+      <c r="B120" s="13" t="n"/>
+    </row>
+    <row r="121">
+      <c r="B121" s="13" t="n"/>
+    </row>
+    <row r="122">
+      <c r="B122" s="13" t="n"/>
+    </row>
+    <row r="123">
+      <c r="B123" s="13" t="n"/>
+    </row>
+    <row r="124">
+      <c r="B124" s="13" t="n"/>
+    </row>
+    <row r="125">
+      <c r="B125" s="13" t="n"/>
+    </row>
+    <row r="126">
+      <c r="B126" s="13" t="n"/>
+    </row>
+    <row r="127">
+      <c r="B127" s="13" t="n"/>
+    </row>
+    <row r="128">
+      <c r="B128" s="13" t="n"/>
+    </row>
+    <row r="129">
+      <c r="B129" s="13" t="n"/>
+    </row>
+    <row r="130">
+      <c r="B130" s="13" t="n"/>
+    </row>
+    <row r="131">
+      <c r="B131" s="13" t="n"/>
+    </row>
+    <row r="132">
+      <c r="B132" s="13" t="n"/>
+    </row>
+    <row r="133">
+      <c r="B133" s="13" t="n"/>
+    </row>
+    <row r="134">
+      <c r="B134" s="13" t="n"/>
+    </row>
+    <row r="135">
+      <c r="B135" s="13" t="n"/>
+    </row>
+    <row r="136">
+      <c r="B136" s="13" t="n"/>
+    </row>
+    <row r="137">
+      <c r="B137" s="13" t="n"/>
+    </row>
+    <row r="138">
+      <c r="B138" s="13" t="n"/>
+    </row>
+    <row r="139">
+      <c r="B139" s="13" t="n"/>
+    </row>
+    <row r="140">
+      <c r="B140" s="13" t="n"/>
+    </row>
+    <row r="141">
+      <c r="B141" s="13" t="n"/>
+    </row>
+    <row r="142">
+      <c r="B142" s="13" t="n"/>
+    </row>
+    <row r="143">
+      <c r="B143" s="13" t="n"/>
+    </row>
+    <row r="144">
+      <c r="B144" s="13" t="n"/>
+    </row>
+    <row r="145">
+      <c r="B145" s="13" t="n"/>
+    </row>
+    <row r="146">
+      <c r="B146" s="13" t="n"/>
+    </row>
+    <row r="147">
+      <c r="B147" s="13" t="n"/>
+    </row>
+    <row r="148">
+      <c r="B148" s="13" t="n"/>
+    </row>
+    <row r="149">
+      <c r="B149" s="13" t="n"/>
+    </row>
+    <row r="150">
+      <c r="B150" s="13" t="n"/>
+    </row>
+    <row r="151">
+      <c r="B151" s="13" t="n"/>
+    </row>
+    <row r="152">
+      <c r="B152" s="13" t="n"/>
+    </row>
+    <row r="153">
+      <c r="B153" s="13" t="n"/>
+    </row>
+    <row r="154">
+      <c r="B154" s="13" t="n"/>
+    </row>
+    <row r="155">
+      <c r="B155" s="13" t="n"/>
+    </row>
+    <row r="156">
+      <c r="B156" s="13" t="n"/>
+    </row>
+    <row r="157">
+      <c r="B157" s="13" t="n"/>
+    </row>
+    <row r="158">
+      <c r="B158" s="13" t="n"/>
+    </row>
+    <row r="159">
+      <c r="B159" s="13" t="n"/>
+    </row>
+    <row r="160">
+      <c r="B160" s="13" t="n"/>
+    </row>
+    <row r="161">
+      <c r="B161" s="13" t="n"/>
+    </row>
+    <row r="162">
+      <c r="B162" s="13" t="n"/>
+    </row>
+    <row r="163">
+      <c r="B163" s="13" t="n"/>
+    </row>
+    <row r="164">
+      <c r="B164" s="13" t="n"/>
+    </row>
+    <row r="165">
+      <c r="B165" s="13" t="n"/>
+    </row>
+    <row r="166">
+      <c r="B166" s="13" t="n"/>
+    </row>
+    <row r="167">
+      <c r="B167" s="13" t="n"/>
+    </row>
+    <row r="168">
+      <c r="B168" s="13" t="n"/>
+    </row>
+    <row r="169">
+      <c r="B169" s="13" t="n"/>
+    </row>
+    <row r="170">
+      <c r="B170" s="13" t="n"/>
+    </row>
+    <row r="171">
+      <c r="B171" s="13" t="n"/>
+    </row>
+    <row r="172">
+      <c r="B172" s="13" t="n"/>
+    </row>
+    <row r="173">
+      <c r="B173" s="13" t="n"/>
+    </row>
+    <row r="174">
+      <c r="B174" s="13" t="n"/>
+    </row>
+    <row r="175">
+      <c r="B175" s="13" t="n"/>
+    </row>
+    <row r="176">
+      <c r="B176" s="13" t="n"/>
+    </row>
+    <row r="177">
+      <c r="B177" s="13" t="n"/>
+    </row>
+    <row r="178">
+      <c r="B178" s="13" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="13" t="n"/>
+    </row>
+    <row r="180">
+      <c r="B180" s="13" t="n"/>
+    </row>
+    <row r="181">
+      <c r="B181" s="13" t="n"/>
+    </row>
+    <row r="182">
+      <c r="B182" s="13" t="n"/>
+    </row>
+    <row r="183">
+      <c r="B183" s="13" t="n"/>
+    </row>
+    <row r="184">
+      <c r="B184" s="13" t="n"/>
+    </row>
+    <row r="185">
+      <c r="B185" s="13" t="n"/>
+    </row>
+    <row r="186">
+      <c r="B186" s="13" t="n"/>
+    </row>
+    <row r="187">
+      <c r="B187" s="13" t="n"/>
+    </row>
+    <row r="188">
+      <c r="B188" s="13" t="n"/>
+    </row>
+    <row r="189">
+      <c r="B189" s="13" t="n"/>
+    </row>
+    <row r="190">
+      <c r="B190" s="13" t="n"/>
+    </row>
+    <row r="191">
+      <c r="B191" s="13" t="n"/>
+    </row>
+    <row r="192">
+      <c r="B192" s="13" t="n"/>
+    </row>
+    <row r="193">
+      <c r="B193" s="13" t="n"/>
+    </row>
+    <row r="194">
+      <c r="B194" s="13" t="n"/>
+    </row>
+    <row r="195">
+      <c r="B195" s="13" t="n"/>
+    </row>
+    <row r="196">
+      <c r="B196" s="13" t="n"/>
+    </row>
+    <row r="197">
+      <c r="B197" s="13" t="n"/>
+    </row>
+    <row r="198">
+      <c r="B198" s="13" t="n"/>
+    </row>
+    <row r="199">
+      <c r="B199" s="13" t="n"/>
+    </row>
+    <row r="200">
+      <c r="B200" s="13" t="n"/>
+    </row>
+    <row r="201">
+      <c r="B201" s="13" t="n"/>
+    </row>
+    <row r="202">
+      <c r="B202" s="13" t="n"/>
+    </row>
+    <row r="203">
+      <c r="B203" s="13" t="n"/>
+    </row>
+    <row r="204">
+      <c r="B204" s="13" t="n"/>
+    </row>
+    <row r="205">
+      <c r="B205" s="13" t="n"/>
+    </row>
+    <row r="206">
+      <c r="B206" s="13" t="n"/>
+    </row>
+    <row r="207">
+      <c r="B207" s="13" t="n"/>
+    </row>
+    <row r="208">
+      <c r="B208" s="13" t="n"/>
+    </row>
+    <row r="209">
+      <c r="B209" s="13" t="n"/>
+    </row>
+    <row r="210">
+      <c r="B210" s="13" t="n"/>
+    </row>
+    <row r="211">
+      <c r="B211" s="13" t="n"/>
+    </row>
+    <row r="212">
+      <c r="B212" s="13" t="n"/>
+    </row>
+    <row r="213">
+      <c r="B213" s="13" t="n"/>
+    </row>
+    <row r="214">
+      <c r="B214" s="13" t="n"/>
+    </row>
+    <row r="215">
+      <c r="B215" s="13" t="n"/>
+    </row>
+    <row r="216">
+      <c r="B216" s="13" t="n"/>
+    </row>
+    <row r="217">
+      <c r="B217" s="13" t="n"/>
+    </row>
+    <row r="218">
+      <c r="B218" s="13" t="n"/>
+    </row>
+    <row r="219">
+      <c r="B219" s="13" t="n"/>
+    </row>
+    <row r="220">
+      <c r="B220" s="13" t="n"/>
+    </row>
+    <row r="221">
+      <c r="B221" s="13" t="n"/>
+    </row>
+    <row r="222">
+      <c r="B222" s="13" t="n"/>
+    </row>
+    <row r="223">
+      <c r="B223" s="13" t="n"/>
+    </row>
+    <row r="224">
+      <c r="B224" s="13" t="n"/>
+    </row>
+    <row r="225">
+      <c r="B225" s="13" t="n"/>
+    </row>
+    <row r="226">
+      <c r="B226" s="13" t="n"/>
+    </row>
+    <row r="227">
+      <c r="B227" s="13" t="n"/>
+    </row>
+    <row r="228">
+      <c r="B228" s="13" t="n"/>
+    </row>
+    <row r="229">
+      <c r="B229" s="13" t="n"/>
+    </row>
+    <row r="230">
+      <c r="B230" s="13" t="n"/>
+    </row>
+    <row r="231">
+      <c r="B231" s="13" t="n"/>
+    </row>
+    <row r="232">
+      <c r="B232" s="13" t="n"/>
+    </row>
+    <row r="233">
+      <c r="B233" s="13" t="n"/>
+    </row>
+    <row r="234">
+      <c r="B234" s="13" t="n"/>
+    </row>
+    <row r="235">
+      <c r="B235" s="13" t="n"/>
+    </row>
+    <row r="236">
+      <c r="B236" s="13" t="n"/>
+    </row>
+    <row r="237">
+      <c r="B237" s="13" t="n"/>
+    </row>
+    <row r="238">
+      <c r="B238" s="13" t="n"/>
+    </row>
+    <row r="239">
+      <c r="B239" s="13" t="n"/>
+    </row>
+    <row r="240">
+      <c r="B240" s="13" t="n"/>
+    </row>
+    <row r="241">
+      <c r="B241" s="13" t="n"/>
+    </row>
+    <row r="242">
+      <c r="B242" s="13" t="n"/>
+    </row>
+    <row r="243">
+      <c r="B243" s="13" t="n"/>
+    </row>
+    <row r="244">
+      <c r="B244" s="13" t="n"/>
+    </row>
+    <row r="245">
+      <c r="B245" s="13" t="n"/>
+    </row>
+    <row r="246">
+      <c r="B246" s="13" t="n"/>
+    </row>
+    <row r="247">
+      <c r="B247" s="13" t="n"/>
+    </row>
+    <row r="248">
+      <c r="B248" s="13" t="n"/>
+    </row>
+    <row r="249">
+      <c r="B249" s="13" t="n"/>
+    </row>
+    <row r="250">
+      <c r="B250" s="13" t="n"/>
+    </row>
+    <row r="251">
+      <c r="B251" s="13" t="n"/>
+    </row>
+    <row r="252">
+      <c r="B252" s="13" t="n"/>
+    </row>
+    <row r="253">
+      <c r="B253" s="13" t="n"/>
+    </row>
+    <row r="254">
+      <c r="B254" s="13" t="n"/>
+    </row>
+    <row r="255">
+      <c r="B255" s="13" t="n"/>
+    </row>
+    <row r="256">
+      <c r="B256" s="13" t="n"/>
+    </row>
+    <row r="257">
+      <c r="B257" s="13" t="n"/>
+    </row>
+    <row r="258">
+      <c r="B258" s="13" t="n"/>
+    </row>
+    <row r="259">
+      <c r="B259" s="13" t="n"/>
+    </row>
+    <row r="260">
+      <c r="B260" s="13" t="n"/>
+    </row>
+    <row r="261">
+      <c r="B261" s="13" t="n"/>
+    </row>
+    <row r="262">
+      <c r="B262" s="13" t="n"/>
+    </row>
+    <row r="263">
+      <c r="B263" s="13" t="n"/>
+    </row>
+    <row r="264">
+      <c r="B264" s="13" t="n"/>
+    </row>
+    <row r="265">
+      <c r="B265" s="13" t="n"/>
+    </row>
+    <row r="266">
+      <c r="B266" s="13" t="n"/>
+    </row>
+    <row r="267">
+      <c r="B267" s="13" t="n"/>
+    </row>
+    <row r="268">
+      <c r="B268" s="13" t="n"/>
+    </row>
+    <row r="269">
+      <c r="B269" s="13" t="n"/>
+    </row>
+    <row r="270">
+      <c r="B270" s="13" t="n"/>
+    </row>
+    <row r="271">
+      <c r="B271" s="13" t="n"/>
+    </row>
+    <row r="272">
+      <c r="B272" s="13" t="n"/>
+    </row>
+    <row r="273">
+      <c r="B273" s="13" t="n"/>
+    </row>
+    <row r="274">
+      <c r="B274" s="13" t="n"/>
+    </row>
+    <row r="275">
+      <c r="B275" s="13" t="n"/>
+    </row>
+    <row r="276">
+      <c r="B276" s="13" t="n"/>
+    </row>
+    <row r="277">
+      <c r="B277" s="13" t="n"/>
+    </row>
+    <row r="278">
+      <c r="B278" s="13" t="n"/>
+    </row>
+    <row r="279">
+      <c r="B279" s="13" t="n"/>
+    </row>
+    <row r="280">
+      <c r="B280" s="13" t="n"/>
+    </row>
+    <row r="281">
+      <c r="B281" s="13" t="n"/>
+    </row>
+    <row r="282">
+      <c r="B282" s="13" t="n"/>
+    </row>
+    <row r="283">
+      <c r="B283" s="13" t="n"/>
+    </row>
+    <row r="284">
+      <c r="B284" s="13" t="n"/>
+    </row>
+    <row r="285">
+      <c r="B285" s="13" t="n"/>
+    </row>
+    <row r="286">
+      <c r="B286" s="13" t="n"/>
+    </row>
+    <row r="287">
+      <c r="B287" s="13" t="n"/>
+    </row>
+    <row r="288">
+      <c r="B288" s="13" t="n"/>
+    </row>
+    <row r="289">
+      <c r="B289" s="13" t="n"/>
+    </row>
+    <row r="290">
+      <c r="B290" s="13" t="n"/>
+    </row>
+    <row r="291">
+      <c r="B291" s="13" t="n"/>
+    </row>
+    <row r="292">
+      <c r="B292" s="13" t="n"/>
+    </row>
+    <row r="293">
+      <c r="B293" s="13" t="n"/>
+    </row>
+    <row r="294">
+      <c r="B294" s="13" t="n"/>
+    </row>
+    <row r="295">
+      <c r="B295" s="13" t="n"/>
+    </row>
+    <row r="296">
+      <c r="B296" s="13" t="n"/>
+    </row>
+    <row r="297">
+      <c r="B297" s="13" t="n"/>
+    </row>
+    <row r="298">
+      <c r="B298" s="13" t="n"/>
+    </row>
+    <row r="299">
+      <c r="B299" s="13" t="n"/>
+    </row>
+    <row r="300">
+      <c r="B300" s="13" t="n"/>
+    </row>
+    <row r="301">
+      <c r="B301" s="13" t="n"/>
+    </row>
+    <row r="302">
+      <c r="B302" s="13" t="n"/>
+    </row>
+    <row r="303">
+      <c r="B303" s="13" t="n"/>
+    </row>
+    <row r="304">
+      <c r="B304" s="13" t="n"/>
+    </row>
+    <row r="305">
+      <c r="B305" s="13" t="n"/>
+    </row>
+    <row r="306">
+      <c r="B306" s="13" t="n"/>
+    </row>
+    <row r="307">
+      <c r="B307" s="13" t="n"/>
+    </row>
+    <row r="308">
+      <c r="B308" s="13" t="n"/>
+    </row>
+    <row r="309">
+      <c r="B309" s="13" t="n"/>
+    </row>
+    <row r="310">
+      <c r="B310" s="13" t="n"/>
+    </row>
+    <row r="311">
+      <c r="B311" s="13" t="n"/>
+    </row>
+    <row r="312">
+      <c r="B312" s="13" t="n"/>
+    </row>
+    <row r="313">
+      <c r="B313" s="13" t="n"/>
+    </row>
+    <row r="314">
+      <c r="B314" s="13" t="n"/>
+    </row>
+    <row r="315">
+      <c r="B315" s="13" t="n"/>
+    </row>
+    <row r="316">
+      <c r="B316" s="13" t="n"/>
+    </row>
+    <row r="317">
+      <c r="B317" s="13" t="n"/>
+    </row>
+    <row r="318">
+      <c r="B318" s="13" t="n"/>
+    </row>
+    <row r="319">
+      <c r="B319" s="13" t="n"/>
+    </row>
+    <row r="320">
+      <c r="B320" s="13" t="n"/>
+    </row>
+    <row r="321">
+      <c r="B321" s="13" t="n"/>
+    </row>
+    <row r="322">
+      <c r="B322" s="13" t="n"/>
+    </row>
+    <row r="323">
+      <c r="B323" s="13" t="n"/>
+    </row>
+    <row r="324">
+      <c r="B324" s="13" t="n"/>
+    </row>
+    <row r="325">
+      <c r="B325" s="13" t="n"/>
+    </row>
+    <row r="326">
+      <c r="B326" s="13" t="n"/>
+    </row>
+    <row r="327">
+      <c r="B327" s="13" t="n"/>
+    </row>
+    <row r="328">
+      <c r="B328" s="13" t="n"/>
+    </row>
+    <row r="329">
+      <c r="B329" s="13" t="n"/>
+    </row>
+    <row r="330">
+      <c r="B330" s="13" t="n"/>
+    </row>
+    <row r="331">
+      <c r="B331" s="13" t="n"/>
+    </row>
+    <row r="332">
+      <c r="B332" s="13" t="n"/>
+    </row>
+    <row r="333">
+      <c r="B333" s="13" t="n"/>
+    </row>
+    <row r="334">
+      <c r="B334" s="13" t="n"/>
+    </row>
+    <row r="335">
+      <c r="B335" s="13" t="n"/>
+    </row>
+    <row r="336">
+      <c r="B336" s="13" t="n"/>
+    </row>
+    <row r="337">
+      <c r="B337" s="13" t="n"/>
+    </row>
+    <row r="338">
+      <c r="B338" s="13" t="n"/>
+    </row>
+    <row r="339">
+      <c r="B339" s="13" t="n"/>
+    </row>
+    <row r="340">
+      <c r="B340" s="13" t="n"/>
+    </row>
+    <row r="341">
+      <c r="B341" s="13" t="n"/>
+    </row>
+    <row r="342">
+      <c r="B342" s="13" t="n"/>
+    </row>
+    <row r="343">
+      <c r="B343" s="13" t="n"/>
+    </row>
+    <row r="344">
+      <c r="B344" s="13" t="n"/>
+    </row>
+    <row r="345">
+      <c r="B345" s="13" t="n"/>
+    </row>
+    <row r="346">
+      <c r="B346" s="13" t="n"/>
+    </row>
+    <row r="347">
+      <c r="B347" s="13" t="n"/>
+    </row>
+    <row r="348">
+      <c r="B348" s="13" t="n"/>
+    </row>
+    <row r="349">
+      <c r="B349" s="13" t="n"/>
+    </row>
+    <row r="350">
+      <c r="B350" s="13" t="n"/>
+    </row>
+    <row r="351">
+      <c r="B351" s="13" t="n"/>
+    </row>
+    <row r="352">
+      <c r="B352" s="13" t="n"/>
+    </row>
+    <row r="353">
+      <c r="B353" s="13" t="n"/>
+    </row>
+    <row r="354">
+      <c r="B354" s="13" t="n"/>
+    </row>
+    <row r="355">
+      <c r="B355" s="13" t="n"/>
+    </row>
+    <row r="356">
+      <c r="B356" s="13" t="n"/>
+    </row>
+    <row r="357">
+      <c r="B357" s="13" t="n"/>
+    </row>
+    <row r="358">
+      <c r="B358" s="13" t="n"/>
+    </row>
+    <row r="359">
+      <c r="B359" s="13" t="n"/>
+    </row>
+    <row r="360">
+      <c r="B360" s="13" t="n"/>
+    </row>
+    <row r="361">
+      <c r="B361" s="13" t="n"/>
+    </row>
+    <row r="362">
+      <c r="B362" s="13" t="n"/>
+    </row>
+    <row r="363">
+      <c r="B363" s="13" t="n"/>
+    </row>
+    <row r="364">
+      <c r="B364" s="13" t="n"/>
+    </row>
+    <row r="365">
+      <c r="B365" s="13" t="n"/>
+    </row>
+    <row r="366">
+      <c r="B366" s="13" t="n"/>
+    </row>
+    <row r="367">
+      <c r="B367" s="13" t="n"/>
+    </row>
+    <row r="368">
+      <c r="B368" s="13" t="n"/>
+    </row>
+    <row r="369">
+      <c r="B369" s="13" t="n"/>
+    </row>
+    <row r="370">
+      <c r="B370" s="13" t="n"/>
+    </row>
+    <row r="371">
+      <c r="B371" s="13" t="n"/>
+    </row>
+    <row r="372">
+      <c r="B372" s="13" t="n"/>
+    </row>
+    <row r="373">
+      <c r="B373" s="13" t="n"/>
+    </row>
+    <row r="374">
+      <c r="B374" s="13" t="n"/>
+    </row>
+    <row r="375">
+      <c r="B375" s="13" t="n"/>
+    </row>
+    <row r="376">
+      <c r="B376" s="13" t="n"/>
+    </row>
+    <row r="377">
+      <c r="B377" s="13" t="n"/>
+    </row>
+    <row r="378">
+      <c r="B378" s="13" t="n"/>
+    </row>
+    <row r="379">
+      <c r="B379" s="13" t="n"/>
+    </row>
+    <row r="380">
+      <c r="B380" s="13" t="n"/>
+    </row>
+    <row r="381">
+      <c r="B381" s="13" t="n"/>
+    </row>
+    <row r="382">
+      <c r="B382" s="13" t="n"/>
+    </row>
+    <row r="383">
+      <c r="B383" s="13" t="n"/>
+    </row>
+    <row r="384">
+      <c r="B384" s="13" t="n"/>
+    </row>
+    <row r="385">
+      <c r="B385" s="13" t="n"/>
+    </row>
+    <row r="386">
+      <c r="B386" s="13" t="n"/>
+    </row>
+    <row r="387">
+      <c r="B387" s="13" t="n"/>
+    </row>
+    <row r="388">
+      <c r="B388" s="13" t="n"/>
+    </row>
+    <row r="389">
+      <c r="B389" s="13" t="n"/>
+    </row>
+    <row r="390">
+      <c r="B390" s="13" t="n"/>
+    </row>
+    <row r="391">
+      <c r="B391" s="13" t="n"/>
+    </row>
+    <row r="392">
+      <c r="B392" s="13" t="n"/>
+    </row>
+    <row r="393">
+      <c r="B393" s="13" t="n"/>
+    </row>
+    <row r="394">
+      <c r="B394" s="13" t="n"/>
+    </row>
+    <row r="395">
+      <c r="B395" s="13" t="n"/>
+    </row>
+    <row r="396">
+      <c r="B396" s="13" t="n"/>
+    </row>
+    <row r="397">
+      <c r="B397" s="13" t="n"/>
+    </row>
+    <row r="398">
+      <c r="B398" s="13" t="n"/>
+    </row>
+    <row r="399">
+      <c r="B399" s="13" t="n"/>
+    </row>
+    <row r="400">
+      <c r="B400" s="13" t="n"/>
+    </row>
+    <row r="401">
+      <c r="B401" s="13" t="n"/>
+    </row>
+    <row r="402">
+      <c r="B402" s="13" t="n"/>
+    </row>
+    <row r="403">
+      <c r="B403" s="13" t="n"/>
+    </row>
+    <row r="404">
+      <c r="B404" s="13" t="n"/>
+    </row>
+    <row r="405">
+      <c r="B405" s="13" t="n"/>
+    </row>
+    <row r="406">
+      <c r="B406" s="13" t="n"/>
+    </row>
+    <row r="407">
+      <c r="B407" s="13" t="n"/>
+    </row>
+    <row r="408">
+      <c r="B408" s="13" t="n"/>
+    </row>
+    <row r="409">
+      <c r="B409" s="13" t="n"/>
+    </row>
+    <row r="410">
+      <c r="B410" s="13" t="n"/>
+    </row>
+    <row r="411">
+      <c r="B411" s="13" t="n"/>
+    </row>
+    <row r="412">
+      <c r="B412" s="13" t="n"/>
+    </row>
+    <row r="413">
+      <c r="B413" s="13" t="n"/>
+    </row>
+    <row r="414">
+      <c r="B414" s="13" t="n"/>
+    </row>
+    <row r="415">
+      <c r="B415" s="13" t="n"/>
+    </row>
+    <row r="416">
+      <c r="B416" s="13" t="n"/>
+    </row>
+    <row r="417">
+      <c r="B417" s="13" t="n"/>
+    </row>
+    <row r="418">
+      <c r="B418" s="13" t="n"/>
+    </row>
+    <row r="419">
+      <c r="B419" s="13" t="n"/>
+    </row>
+    <row r="420">
+      <c r="B420" s="13" t="n"/>
+    </row>
+    <row r="421">
+      <c r="B421" s="13" t="n"/>
+    </row>
+    <row r="422">
+      <c r="B422" s="13" t="n"/>
+    </row>
+    <row r="423">
+      <c r="B423" s="13" t="n"/>
+    </row>
+    <row r="424">
+      <c r="B424" s="13" t="n"/>
+    </row>
+    <row r="425">
+      <c r="B425" s="13" t="n"/>
+    </row>
+    <row r="426">
+      <c r="B426" s="13" t="n"/>
+    </row>
+    <row r="427">
+      <c r="B427" s="13" t="n"/>
+    </row>
+    <row r="428">
+      <c r="B428" s="13" t="n"/>
+    </row>
+    <row r="429">
+      <c r="B429" s="13" t="n"/>
+    </row>
+    <row r="430">
+      <c r="B430" s="13" t="n"/>
+    </row>
+    <row r="431">
+      <c r="B431" s="13" t="n"/>
+    </row>
+    <row r="432">
+      <c r="B432" s="13" t="n"/>
+    </row>
+    <row r="433">
+      <c r="B433" s="13" t="n"/>
+    </row>
+    <row r="434">
+      <c r="B434" s="13" t="n"/>
+    </row>
+    <row r="435">
+      <c r="B435" s="13" t="n"/>
+    </row>
+    <row r="436">
+      <c r="B436" s="13" t="n"/>
+    </row>
+    <row r="437">
+      <c r="B437" s="13" t="n"/>
+    </row>
+    <row r="438">
+      <c r="B438" s="13" t="n"/>
+    </row>
+    <row r="439">
+      <c r="B439" s="13" t="n"/>
+    </row>
+    <row r="440">
+      <c r="B440" s="13" t="n"/>
+    </row>
+    <row r="441">
+      <c r="B441" s="13" t="n"/>
+    </row>
+    <row r="442">
+      <c r="B442" s="13" t="n"/>
+    </row>
+    <row r="443">
+      <c r="B443" s="13" t="n"/>
+    </row>
+    <row r="444">
+      <c r="B444" s="13" t="n"/>
+    </row>
+    <row r="445">
+      <c r="B445" s="13" t="n"/>
+    </row>
+    <row r="446">
+      <c r="B446" s="13" t="n"/>
+    </row>
+    <row r="447">
+      <c r="B447" s="13" t="n"/>
+    </row>
+    <row r="448">
+      <c r="B448" s="13" t="n"/>
+    </row>
+    <row r="449">
+      <c r="B449" s="13" t="n"/>
+    </row>
+    <row r="450">
+      <c r="B450" s="13" t="n"/>
+    </row>
+    <row r="451">
+      <c r="B451" s="13" t="n"/>
+    </row>
+    <row r="452">
+      <c r="B452" s="13" t="n"/>
+    </row>
+    <row r="453">
+      <c r="B453" s="13" t="n"/>
+    </row>
+    <row r="454">
+      <c r="B454" s="13" t="n"/>
+    </row>
+    <row r="455">
+      <c r="B455" s="13" t="n"/>
+    </row>
+    <row r="456">
+      <c r="B456" s="13" t="n"/>
+    </row>
+    <row r="457">
+      <c r="B457" s="13" t="n"/>
+    </row>
+    <row r="458">
+      <c r="B458" s="13" t="n"/>
+    </row>
+    <row r="459">
+      <c r="B459" s="13" t="n"/>
+    </row>
+    <row r="460">
+      <c r="B460" s="13" t="n"/>
+    </row>
+    <row r="461">
+      <c r="B461" s="13" t="n"/>
+    </row>
+    <row r="462">
+      <c r="B462" s="13" t="n"/>
+    </row>
+    <row r="463">
+      <c r="B463" s="13" t="n"/>
+    </row>
+    <row r="464">
+      <c r="B464" s="13" t="n"/>
+    </row>
+    <row r="465">
+      <c r="B465" s="13" t="n"/>
+    </row>
+    <row r="466">
+      <c r="B466" s="13" t="n"/>
+    </row>
+    <row r="467">
+      <c r="B467" s="13" t="n"/>
+    </row>
+    <row r="468">
+      <c r="B468" s="13" t="n"/>
+    </row>
+    <row r="469">
+      <c r="B469" s="13" t="n"/>
+    </row>
+    <row r="470">
+      <c r="B470" s="13" t="n"/>
+    </row>
+    <row r="471">
+      <c r="B471" s="13" t="n"/>
+    </row>
+    <row r="472">
+      <c r="B472" s="13" t="n"/>
+    </row>
+    <row r="473">
+      <c r="B473" s="13" t="n"/>
+    </row>
+    <row r="474">
+      <c r="B474" s="13" t="n"/>
+    </row>
+    <row r="475">
+      <c r="B475" s="13" t="n"/>
+    </row>
+    <row r="476">
+      <c r="B476" s="13" t="n"/>
+    </row>
+    <row r="477">
+      <c r="B477" s="13" t="n"/>
+    </row>
+    <row r="478">
+      <c r="B478" s="13" t="n"/>
+    </row>
+    <row r="479">
+      <c r="B479" s="13" t="n"/>
+    </row>
+    <row r="480">
+      <c r="B480" s="13" t="n"/>
+    </row>
+    <row r="481">
+      <c r="B481" s="13" t="n"/>
+    </row>
+    <row r="482">
+      <c r="B482" s="13" t="n"/>
+    </row>
+    <row r="483">
+      <c r="B483" s="13" t="n"/>
+    </row>
+    <row r="484">
+      <c r="B484" s="13" t="n"/>
+    </row>
+    <row r="485">
+      <c r="B485" s="13" t="n"/>
+    </row>
+    <row r="486">
+      <c r="B486" s="13" t="n"/>
+    </row>
+    <row r="487">
+      <c r="B487" s="13" t="n"/>
+    </row>
+    <row r="488">
+      <c r="B488" s="13" t="n"/>
+    </row>
+    <row r="489">
+      <c r="B489" s="13" t="n"/>
+    </row>
+    <row r="490">
+      <c r="B490" s="13" t="n"/>
+    </row>
+    <row r="491">
+      <c r="B491" s="13" t="n"/>
+    </row>
+    <row r="492">
+      <c r="B492" s="13" t="n"/>
+    </row>
+    <row r="493">
+      <c r="B493" s="13" t="n"/>
+    </row>
+    <row r="494">
+      <c r="B494" s="13" t="n"/>
+    </row>
+    <row r="495">
+      <c r="B495" s="13" t="n"/>
+    </row>
+    <row r="496">
+      <c r="B496" s="13" t="n"/>
+    </row>
+    <row r="497">
+      <c r="B497" s="13" t="n"/>
+    </row>
+    <row r="498">
+      <c r="B498" s="13" t="n"/>
+    </row>
+    <row r="499">
+      <c r="B499" s="13" t="n"/>
+    </row>
+    <row r="500">
+      <c r="B500" s="13" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>